<commit_message>
Quota di sgombero all'inversione configurabile per passata
Il punto in cui il pezzo si ferma per invertire era il risultato della distanza
di frenata dell'azionamento invece che un dato di processo. Ora e' la colonna
reversing_clearance_m: il pezzo prosegue e frena per fermarsi esattamente li',
e se la quota richiesta e' piu' corta della distanza di frenata il tool riporta
quella ottenuta invece di fingere una frenata impossibile.

Pesa parecchio: sull'esempio, da 0 a 20 m di sgombero il pacing minimo passa da
105 a 149 secondi.

Aggiunta anche la regola mancante che rifiuta una schedule terminante con una
passata inversa, e la tolleranza alle colonne opzionali nel lettore Excel, cosi'
un workbook compilato prima resta valido.

Co-authored-by: giacomofm <giacomofm@gmail.com>
</commit_message>
<xml_diff>
--- a/examples/hsm_example.xlsx
+++ b/examples/hsm_example.xlsx
@@ -463,25 +463,30 @@
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
+        <t>Distanza fra gabbia ed estremita' piu' vicina alla fermata per invertire, m (vuoto = minima distanza di frenata)</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
         <t>Velocita' di avvicinamento dopo l'inversione (vuoto = v_ingresso)</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>SI sulla gabbia che detta il bilancio di massa del gruppo tandem</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>Zoom rolling: incremento di velocita' in %</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>Zoom: avanzamento della testa virtuale oltre questa gabbia, m</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>Zoom: accelerazione, m/s2 (vuoto = quella dell'asse)</t>
       </text>
@@ -804,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -892,42 +897,49 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
+    <row r="15" ht="75" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Dopo il tail-out il pezzo decelera fino a fermarsi, attende il reversing delay della passata successiva e riparte nel verso opposto. Il reversing delay deve gia' comprendere screwdown e centraggio sideguides.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+          <t>Dopo il tail-out il pezzo prosegue fino a portare l'estremita' piu' vicina alla gabbia a reversing_clearance_m metri da essa, dove si ferma, attende il reversing delay della passata successiva e riparte nel verso opposto. Il reversing delay deve gia' comprendere screwdown e centraggio sideguides, e la quota di sgombero va misurata dalla gabbia, quindi va aumentata se il vincolo vero e' l'edger che sta qualche metro prima.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Lasciando vuota la quota di sgombero il pezzo si ferma appena la decelerazione lo consente, cioe' a v^2/(2a) dalla gabbia. Se la quota richiesta e' piu' corta di quella distanza il tool lo segnala invece di fingere una frenata impossibile.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Zoom rolling</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Definito come incremento percentuale di velocita' che parte quando la testa ha superato di zoom_trigger_m la gabbia indicata. Il trigger usa la testa virtuale, cioe' ignora il fatto che la testa si ferma all'avvolgitore: se il trigger cade oltre l'avvolgitore lo zoom parte dopo qualche avvolgimento, come nel modello offline.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Cosa il modello non fa</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Nessun interblocco e nessun hold point: i pezzi seguono i profili nominali e il tool riporta dove il gap scende sotto soglia, senza fermare il pezzo che segue. Slittamento sui rulli trascurato, jerk infinito, nessun modello termico, nessun vincolo di forno o di ciclo avvolgitore.</t>
         </is>
@@ -1929,7 +1941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1942,11 +1954,12 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="23" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="23" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2002,25 +2015,30 @@
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
+          <t>reversing_clearance_m</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
           <t>approach_v_mps</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>master</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>zoom_pct</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>zoom_trigger_m</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>zoom_accel_mps2</t>
         </is>
@@ -2063,7 +2081,7 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2102,7 +2120,10 @@
       <c r="J3" t="n">
         <v>6</v>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2141,7 +2162,10 @@
       <c r="J4" t="n">
         <v>6</v>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="K4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2180,7 +2204,7 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2219,7 +2243,10 @@
       <c r="J6" t="n">
         <v>6</v>
       </c>
-      <c r="L6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2258,7 +2285,10 @@
       <c r="J7" t="n">
         <v>6</v>
       </c>
-      <c r="L7" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2297,7 +2327,7 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2336,7 +2366,7 @@
       <c r="J9" t="n">
         <v>0</v>
       </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2375,7 +2405,7 @@
       <c r="J10" t="n">
         <v>0</v>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2414,7 +2444,7 @@
       <c r="J11" t="n">
         <v>0</v>
       </c>
-      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2453,7 +2483,7 @@
       <c r="J12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2492,7 +2522,7 @@
       <c r="J13" t="n">
         <v>0</v>
       </c>
-      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2531,15 +2561,15 @@
       <c r="J14" t="n">
         <v>0</v>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="M14" t="n">
+      <c r="N14" t="n">
         <v>8</v>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>130</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Translate the whole project to English
Interface, code comments and docstrings, validation and error messages, Excel
template and guide sheet, result sheet names, chart labels, CLI help and
output, test names, README and documents. Only the conversation with the user
stays in Italian.

Also fixed the plural in the validation error header.

Co-authored-by: giacomofm <giacomofm@gmail.com>
</commit_message>
<xml_diff>
--- a/examples/hsm_example.xlsx
+++ b/examples/hsm_example.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Guida" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Guide" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Info" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Layout" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Sections" sheetId="4" state="visible" r:id="rId4"/>
@@ -163,12 +163,12 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Chiave</t>
+        <t>Key</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Valore</t>
+        <t>Value</t>
       </text>
     </comment>
   </commentList>
@@ -183,7 +183,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Identificativo univoco (R1, F7, DC1)</t>
+        <t>Unique identifier (R1, F7, DC1)</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -193,22 +193,22 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Posizione assoluta lungo la linea, in metri</t>
+        <t>Absolute position along the line, in metres</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Accelerazione = decelerazione dell'asse, m/s2</t>
+        <t>Acceleration = deceleration of the axis, m/s2</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Gruppo tandem, es. FM per le gabbie finitrici</t>
+        <t>Tandem group, for example FM for the finishing stands</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Descrizione mostrata sui grafici</t>
+        <t>Description shown on the charts</t>
       </text>
     </comment>
   </commentList>
@@ -223,142 +223,142 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Identificativo univoco della sezione</t>
+        <t>Unique identifier of the section</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Descrizione mostrata sui grafici</t>
+        <t>Description shown on the charts</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Apparecchiatura di riferimento, 'prev' o vuoto per assoluto</t>
+        <t>Reference equipment, 'prev', or empty for an absolute position</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Distanza dal riferimento all'inizio della sezione, m</t>
+        <t>Distance from the reference to the start of the section, m</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Lunghezza della sezione, m</t>
+        <t>Length of the section, m</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>fwd | rev: verso di moto in cui gli eventi sono validi</t>
+        <t>fwd | rev: direction of travel in which the events apply</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>SI se l'evento vale anche in laminazione, NO per differirlo</t>
+        <t>YES if the event applies while rolling, NO to defer it</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Distanza dall'inizio sezione del cambio di velocita' 1, m</t>
+        <t>Distance from the start of the section of speed change 1, m</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Nuova velocita' comandata 1, m/s</t>
+        <t>New commanded speed 1, m/s</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Accelerazione del cambio 1, m/s2 (vuoto = quella dell'asse)</t>
+        <t>Acceleration of change 1, m/s2 (empty = the one of the axis)</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Distanza dall'inizio sezione del cambio di velocita' 2, m</t>
+        <t>Distance from the start of the section of speed change 2, m</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>Nuova velocita' comandata 2, m/s</t>
+        <t>New commanded speed 2, m/s</t>
       </text>
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>Accelerazione del cambio 2, m/s2 (vuoto = quella dell'asse)</t>
+        <t>Acceleration of change 2, m/s2 (empty = the one of the axis)</t>
       </text>
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>Distanza dall'inizio sezione del cambio di velocita' 3, m</t>
+        <t>Distance from the start of the section of speed change 3, m</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
-        <t>Nuova velocita' comandata 3, m/s</t>
+        <t>New commanded speed 3, m/s</t>
       </text>
     </comment>
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
-        <t>Accelerazione del cambio 3, m/s2 (vuoto = quella dell'asse)</t>
+        <t>Acceleration of change 3, m/s2 (empty = the one of the axis)</t>
       </text>
     </comment>
     <comment ref="Q1" authorId="0" shapeId="0">
       <text>
-        <t>Distanza dall'inizio sezione del cambio di velocita' 4, m</t>
+        <t>Distance from the start of the section of speed change 4, m</t>
       </text>
     </comment>
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
-        <t>Nuova velocita' comandata 4, m/s</t>
+        <t>New commanded speed 4, m/s</t>
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
       <text>
-        <t>Accelerazione del cambio 4, m/s2 (vuoto = quella dell'asse)</t>
+        <t>Acceleration of change 4, m/s2 (empty = the one of the axis)</t>
       </text>
     </comment>
     <comment ref="T1" authorId="0" shapeId="0">
       <text>
-        <t>Distanza dall'inizio sezione del cambio di velocita' 5, m</t>
+        <t>Distance from the start of the section of speed change 5, m</t>
       </text>
     </comment>
     <comment ref="U1" authorId="0" shapeId="0">
       <text>
-        <t>Nuova velocita' comandata 5, m/s</t>
+        <t>New commanded speed 5, m/s</t>
       </text>
     </comment>
     <comment ref="V1" authorId="0" shapeId="0">
       <text>
-        <t>Accelerazione del cambio 5, m/s2 (vuoto = quella dell'asse)</t>
+        <t>Acceleration of change 5, m/s2 (empty = the one of the axis)</t>
       </text>
     </comment>
     <comment ref="W1" authorId="0" shapeId="0">
       <text>
-        <t>Distanza dall'inizio sezione del cambio di velocita' 6, m</t>
+        <t>Distance from the start of the section of speed change 6, m</t>
       </text>
     </comment>
     <comment ref="X1" authorId="0" shapeId="0">
       <text>
-        <t>Nuova velocita' comandata 6, m/s</t>
+        <t>New commanded speed 6, m/s</t>
       </text>
     </comment>
     <comment ref="Y1" authorId="0" shapeId="0">
       <text>
-        <t>Accelerazione del cambio 6, m/s2 (vuoto = quella dell'asse)</t>
+        <t>Acceleration of change 6, m/s2 (empty = the one of the axis)</t>
       </text>
     </comment>
     <comment ref="Z1" authorId="0" shapeId="0">
       <text>
-        <t>Distanza dall'inizio sezione del cambio di velocita' 7, m</t>
+        <t>Distance from the start of the section of speed change 7, m</t>
       </text>
     </comment>
     <comment ref="AA1" authorId="0" shapeId="0">
       <text>
-        <t>Nuova velocita' comandata 7, m/s</t>
+        <t>New commanded speed 7, m/s</t>
       </text>
     </comment>
     <comment ref="AB1" authorId="0" shapeId="0">
       <text>
-        <t>Accelerazione del cambio 7, m/s2 (vuoto = quella dell'asse)</t>
+        <t>Acceleration of change 7, m/s2 (empty = the one of the axis)</t>
       </text>
     </comment>
   </commentList>
@@ -373,32 +373,32 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Identificativo univoco del prodotto</t>
+        <t>Unique identifier of the product</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Descrizione</t>
+        <t>Description</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Qualita' acciaio</t>
+        <t>Steel grade</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Spessore bramma, mm</t>
+        <t>Slab thickness, mm</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Larghezza bramma, mm</t>
+        <t>Slab width, mm</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Lunghezza bramma, m</t>
+        <t>Slab length, m</t>
       </text>
     </comment>
   </commentList>
@@ -413,17 +413,17 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Prodotto a cui appartiene la passata</t>
+        <t>Product this pass belongs to</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Numero d'ordine della passata</t>
+        <t>Sequence number of the pass</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Gabbia su cui avviene la passata</t>
+        <t>Stand where the pass takes place</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
@@ -433,62 +433,62 @@
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Spessore in ingresso, mm</t>
+        <t>Entry thickness, mm</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Spessore in uscita, mm</t>
+        <t>Exit thickness, mm</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Larghezza in ingresso, mm</t>
+        <t>Entry width, mm</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Larghezza in uscita, mm</t>
+        <t>Exit width, mm</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Velocita' del materiale in uscita gabbia, m/s</t>
+        <t>Material speed at the stand exit, m/s</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Tempo morto prima di questa passata se cambia il verso, s</t>
+        <t>Dead time ahead of this pass when the direction changes, s</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Distanza fra gabbia ed estremita' piu' vicina alla fermata per invertire, m (vuoto = minima distanza di frenata)</t>
+        <t>Distance between the stand and the closest extremity when the piece stops to reverse, m (empty = shortest braking distance)</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>Velocita' di avvicinamento dopo l'inversione (vuoto = v_ingresso)</t>
+        <t>Approach speed after the reversal (empty = entry speed)</t>
       </text>
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>SI sulla gabbia che detta il bilancio di massa del gruppo tandem</t>
+        <t>YES on the stand that sets the mass flow of the tandem group</t>
       </text>
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>Zoom rolling: incremento di velocita' in %</t>
+        <t>Zoom rolling: speed increase in per cent</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
-        <t>Zoom: avanzamento della testa virtuale oltre questa gabbia, m</t>
+        <t>Zoom: travel of the virtual head beyond this stand, m</t>
       </text>
     </comment>
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
-        <t>Zoom: accelerazione, m/s2 (vuoto = quella dell'asse)</t>
+        <t>Zoom: acceleration, m/s2 (empty = the one of the axis)</t>
       </text>
     </comment>
   </commentList>
@@ -503,17 +503,17 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Chiave</t>
+        <t>Key</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Valore</t>
+        <t>Value</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Descrizione</t>
+        <t>Description</t>
       </text>
     </comment>
   </commentList>
@@ -818,7 +818,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Come e' fatto il modello</t>
+          <t>How the model works</t>
         </is>
       </c>
     </row>
@@ -828,14 +828,14 @@
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>La testa comanda, la coda si deduce. Si descrivono i cambi di velocita' dell'estremita' che guida nel verso corrente; la velocita' dell'altra estremita' discende dal bilancio di massa delle gabbie ingaggiate:</t>
+          <t>The head commands, the tail follows. You describe the speed changes of the extremity that leads in the current direction of travel; the speed of the other extremity follows from the mass flow balance of the engaged stands:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    v_trascinata = v_guida / prodotto dei lambda,   lambda = (h_in*w_in)/(h_out*w_out)</t>
+          <t xml:space="preserve">    v_trailing = v_leading / product of the lambdas,   lambda = (h_in*w_in)/(h_out*w_out)</t>
         </is>
       </c>
     </row>
@@ -845,21 +845,21 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Unita' fissate nel file, nessuna colonna unita' da compilare:</t>
+          <t>Units are fixed in the file, there is no unit column to fill in:</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    posizioni e lunghezze in m, spessori e larghezze in mm,</t>
+          <t xml:space="preserve">    positions and lengths in m, thicknesses and widths in mm,</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    velocita' in m/s, tempi in s, accelerazioni in m/s2.</t>
+          <t xml:space="preserve">    speeds in m/s, times in s, accelerations in m/s2.</t>
         </is>
       </c>
     </row>
@@ -869,21 +869,21 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Sezioni ed eventi di velocita'</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
+          <t>Sections and speed events</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Le vie a rulli non hanno un setpoint proprio: la linea e' divisa in sezioni definite da chi compila, anche piu' corte dell'interasse fra due gabbie. Ogni sezione ammette fino a 7 cambi di velocita', dati come distanza dall'inizio della sezione piu' velocita' obiettivo.</t>
+          <t>Roller tables have no setpoint of their own: the line is divided into sections defined by whoever fills in the file, possibly shorter than the spacing between two stands. Each section allows up to 7 speed changes, given as a distance from the start of the section plus a target speed.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Un evento che scatta mentre una passata e' ingaggiata viene differito al disingaggio, perche' in laminazione comanda il mill e non la via a rulli. Mettere SI in during_pass per farlo valere comunque.</t>
+          <t>An event that would fire while a pass is engaged is deferred to disengagement, because while rolling it is the mill that commands, not the roller table. Put YES in during_pass to make it apply anyway.</t>
         </is>
       </c>
     </row>
@@ -893,21 +893,21 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Sbozzatura reversibile</t>
+          <t>Reversing roughing</t>
         </is>
       </c>
     </row>
     <row r="15" ht="75" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Dopo il tail-out il pezzo prosegue fino a portare l'estremita' piu' vicina alla gabbia a reversing_clearance_m metri da essa, dove si ferma, attende il reversing delay della passata successiva e riparte nel verso opposto. Il reversing delay deve gia' comprendere screwdown e centraggio sideguides, e la quota di sgombero va misurata dalla gabbia, quindi va aumentata se il vincolo vero e' l'edger che sta qualche metro prima.</t>
+          <t>After tail-out the piece keeps going until the extremity closest to the stand is reversing_clearance_m metres away from it, where it stops, waits for the reversing delay of the following pass and restarts in the opposite direction. The reversing delay must already include screwdown and side guide centring, and the clearance is measured from the stand, so increase it if the real constraint is the edger a few metres before.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lasciando vuota la quota di sgombero il pezzo si ferma appena la decelerazione lo consente, cioe' a v^2/(2a) dalla gabbia. Se la quota richiesta e' piu' corta di quella distanza il tool lo segnala invece di fingere una frenata impossibile.</t>
+          <t>Leaving the clearance empty makes the piece stop as soon as the deceleration allows, that is at v^2/(2a) from the stand. If the requested clearance is shorter than that distance the tool reports it rather than faking an impossible braking.</t>
         </is>
       </c>
     </row>
@@ -924,7 +924,7 @@
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Definito come incremento percentuale di velocita' che parte quando la testa ha superato di zoom_trigger_m la gabbia indicata. Il trigger usa la testa virtuale, cioe' ignora il fatto che la testa si ferma all'avvolgitore: se il trigger cade oltre l'avvolgitore lo zoom parte dopo qualche avvolgimento, come nel modello offline.</t>
+          <t>Defined as a percentage speed increase starting when the head has travelled zoom_trigger_m beyond the given stand. The trigger uses the virtual head, that is it ignores the fact that the head stops at the coiler: if the trigger falls beyond the coiler the zoom starts after a few wraps, as in the offline model.</t>
         </is>
       </c>
     </row>
@@ -934,14 +934,14 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Cosa il modello non fa</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1">
+          <t>What the model does not do</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Nessun interblocco e nessun hold point: i pezzi seguono i profili nominali e il tool riporta dove il gap scende sotto soglia, senza fermare il pezzo che segue. Slittamento sui rulli trascurato, jerk infinito, nessun modello termico, nessun vincolo di forno o di ciclo avvolgitore.</t>
+          <t>No interlocks and no hold points: the pieces follow their nominal profiles and the tool reports where the gap drops below the threshold, without stopping the piece behind. Roller slip neglected, infinite jerk, no thermal model, no furnace or coiler cycle constraint.</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HSM di esempio</t>
+          <t>Example HSM</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dati inventati a scopo dimostrativo</t>
+          <t>Invented data, for demonstration only</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Uscita forno</t>
+          <t>Furnace exit</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Descagliatore primario</t>
+          <t>Primary descaler</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Sbozzatore R1</t>
+          <t>Roughing stand R1</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Sbozzatore R2</t>
+          <t>Roughing stand R2</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Cesoia crop</t>
+          <t>Crop shear</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Descagliatore finitore</t>
+          <t>Finishing descaler</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Avvolgitore 1</t>
+          <t>Downcoiler 1</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Forno - R1</t>
+          <t>Furnace to R1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R1 - R2</t>
+          <t>R1 to R2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tavolo di trasferimento</t>
+          <t>Transfer table</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cesoia - F1</t>
+          <t>Shear to F1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Finitore - avvolgitore</t>
+          <t>Finishing mill to coiler</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="N14" t="n">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Cadenza nominale fra un pezzo e il successivo, s</t>
+          <t>Nominal cadence between one piece and the next, s</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Numero di pezzi simulati</t>
+          <t>Number of simulated pieces</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
       <c r="B4" t="inlineStr"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Sequenza prodotti separata da virgole (vuoto = ripete il primo)</t>
+          <t>Comma separated product sequence (empty = repeat the first)</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Distanza minima ammessa fra coda e testa successiva, m</t>
+          <t>Minimum distance allowed between a tail and the next head, m</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Estremo inferiore della scansione del pacing, s</t>
+          <t>Lower bound of the pacing scan, s</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Estremo superiore della scansione del pacing, s</t>
+          <t>Upper bound of the pacing scan, s</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Numero di punti della scansione</t>
+          <t>Number of points in the scan</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Numero di run Monte Carlo per la robustezza</t>
+          <t>Number of Monte Carlo runs for the robustness study</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Tolleranza sulle velocita' di passata, +/- %</t>
+          <t>Tolerance on the pass speeds, +/- %</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Deviazione standard sui tempi morti, s</t>
+          <t>Standard deviation of the dead times, s</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Deviazione standard sull'istante di rilascio, s</t>
+          <t>Standard deviation of the release instant, s</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Seme del generatore casuale, per risultati riproducibili</t>
+          <t>Seed of the random generator, for reproducible results</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Tempo massimo di simulazione di un pezzo, s</t>
+          <t>Maximum simulation time of a single piece, s</t>
         </is>
       </c>
     </row>
@@ -2811,12 +2811,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>SI per tempo crescente verso il basso nel diagramma</t>
+          <t>YES for time increasing downwards on the diagram</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Blank the dead reversal cells in the workbook and record the second review round
Co-authored-by: giacomofm <giacomofm@gmail.com>
</commit_message>
<xml_diff>
--- a/examples/hsm_example.xlsx
+++ b/examples/hsm_example.xlsx
@@ -2300,9 +2300,6 @@
       <c r="I4" t="n">
         <v>3.5</v>
       </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
       <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -2423,9 +2420,6 @@
       <c r="I7" t="n">
         <v>4.5</v>
       </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
       <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -2462,9 +2456,6 @@
       <c r="I8" t="n">
         <v>1.7</v>
       </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
       <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -2501,9 +2492,6 @@
       <c r="I9" t="n">
         <v>2.84</v>
       </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
       <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -2540,9 +2528,6 @@
       <c r="I10" t="n">
         <v>4.36</v>
       </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
       <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -2579,9 +2564,6 @@
       <c r="I11" t="n">
         <v>6.25</v>
       </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
       <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
@@ -2618,9 +2600,6 @@
       <c r="I12" t="n">
         <v>8.33</v>
       </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
       <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -2657,9 +2636,6 @@
       <c r="I13" t="n">
         <v>10.42</v>
       </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
       <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -2695,9 +2671,6 @@
       </c>
       <c r="I14" t="n">
         <v>12.5</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>

</xml_diff>